<commit_message>
feat(data): erase legacy items and generate fresh high-spec CPSE catalogs
</commit_message>
<xml_diff>
--- a/frontend/public/catalogs/BPCL_Procurement_Master_2026.xlsx
+++ b/frontend/public/catalogs/BPCL_Procurement_Master_2026.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Material Catalog" sheetId="1" r:id="rId1"/>
+    <sheet name="BPCL_Materials" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -421,110 +421,110 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BPCL-MAT-PIPE-640</v>
+        <v>BPCL-INST-PDT-250MB</v>
       </c>
       <c r="B2" t="str">
-        <v>Seamless CS Pipe 6 inch NB Schedule 40 ASTM A106 Grade B Beveled</v>
+        <v>Diff. Pressure Transmitter 4-20mA HART Communication 0-250 mbar Hastelloy-C Diaphragm Ex-Proof</v>
       </c>
       <c r="C2" t="str">
-        <v>Pipes</v>
+        <v>Instrumentation</v>
       </c>
       <c r="D2" t="str">
-        <v>Mtr</v>
+        <v>Nos</v>
       </c>
       <c r="E2">
-        <v>4920</v>
+        <v>78900</v>
       </c>
       <c r="F2">
-        <v>10500</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>BPCL-MAT-PIPE-440</v>
+        <v>BPCL-VAL-BFLY-8150</v>
       </c>
       <c r="B3" t="str">
-        <v>Carbon Steel Seamless Pipe 4" NB Sch 40 to ASTM A106 Gr B</v>
+        <v>Valve Butterfly 8" 150# Lugged Metal to Metal Seat WCB Body SS316 Disc API 609 Cat B Handwheel / Gear Operated</v>
       </c>
       <c r="C3" t="str">
-        <v>Pipes</v>
+        <v>Valves</v>
       </c>
       <c r="D3" t="str">
-        <v>Mtr</v>
+        <v>Nos</v>
       </c>
       <c r="E3">
-        <v>3250</v>
+        <v>64500</v>
       </c>
       <c r="F3">
-        <v>7200</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BPCL-PIP-SS316-02</v>
+        <v>BPCL-INST-COR-50K</v>
       </c>
       <c r="B4" t="str">
-        <v>Stainless Steel Pipe 2" NB Seamless Sch 40S ASTM A312 Grade TP316L</v>
+        <v>Coriolis Mass Flow Meter Size 50mm (2") Flange 300# SS316L Body Accuracy 0.1% Mass Rate 50 T/hr with Local Display</v>
       </c>
       <c r="C4" t="str">
-        <v>Pipes</v>
+        <v>Instrumentation</v>
       </c>
       <c r="D4" t="str">
-        <v>Mtr</v>
+        <v>Nos</v>
       </c>
       <c r="E4">
-        <v>8950</v>
+        <v>322000</v>
       </c>
       <c r="F4">
-        <v>3800</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>BPCL-VAL-BALL-304</v>
+        <v>BPCL-MAT-LTCS-880</v>
       </c>
       <c r="B5" t="str">
-        <v>Valve Ball Flanged 4 inch 300# Full Port CS A216 WCB RF Lever Operated</v>
+        <v>Carbon Steel Pipe Seamless Low Temp Grade 6 ASTM A333 8" NB Sch 80 Plain / Beveled</v>
       </c>
       <c r="C5" t="str">
-        <v>Valves</v>
+        <v>Pipes</v>
       </c>
       <c r="D5" t="str">
-        <v>Nos</v>
+        <v>Mtr</v>
       </c>
       <c r="E5">
-        <v>24900</v>
+        <v>14180</v>
       </c>
       <c r="F5">
-        <v>390</v>
+        <v>5800</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>BPCL-VAL-GATE-156</v>
+        <v>BPCL-INST-RTD-100D</v>
       </c>
       <c r="B6" t="str">
-        <v>Gate Valve 6" 150# Flanged WCB Body Bolted Bonnet Trim 8 to API 600</v>
+        <v>Pt100 Resistance Temperature Detector Duplex 3 Wire SS316 Sheath L=400mm with Thermowell Flange 1-1/2 Inch 300#</v>
       </c>
       <c r="C6" t="str">
-        <v>Valves</v>
+        <v>Instrumentation</v>
       </c>
       <c r="D6" t="str">
         <v>Nos</v>
       </c>
       <c r="E6">
-        <v>38500</v>
+        <v>12600</v>
       </c>
       <c r="F6">
-        <v>290</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>BPCL-VAL-CHCK-303</v>
+        <v>BPCL-VAL-NDL-05-6M</v>
       </c>
       <c r="B7" t="str">
-        <v>Check Valve Swing Type 3 inch Class 300 RF Flanged WCB API 6D</v>
+        <v>Valve Needle 1/2" NPT Female 6000# Pressure SS316 Construction High Pressure Gauge Isolation</v>
       </c>
       <c r="C7" t="str">
         <v>Valves</v>
@@ -533,290 +533,290 @@
         <v>Nos</v>
       </c>
       <c r="E7">
-        <v>16800</v>
+        <v>4250</v>
       </c>
       <c r="F7">
-        <v>240</v>
+        <v>780</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>BPCL-VAL-GLOB-302</v>
+        <v>BPCL-FLG-SPBL-8300</v>
       </c>
       <c r="B8" t="str">
-        <v>Globe Valve 2 inch Class 300 Flanged WCB Body OS&amp;Y Stem to BS 1873</v>
+        <v>Figure 8 Spectacle Blind 8" 300# RF Carbon Steel Plate A516 Gr.70 ASME B16.48</v>
       </c>
       <c r="C8" t="str">
-        <v>Valves</v>
+        <v>Fittings</v>
       </c>
       <c r="D8" t="str">
         <v>Nos</v>
       </c>
       <c r="E8">
-        <v>14400</v>
+        <v>8500</v>
       </c>
       <c r="F8">
-        <v>310</v>
+        <v>290</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>BPCL-BLT-ST-2012</v>
+        <v>BPCL-GSK-RING-R45</v>
       </c>
       <c r="B9" t="str">
-        <v>Stud Bolt 20mm Dia x 120mm Long Alloy Steel A193-B7 with 2H Hex Nuts</v>
+        <v>RTJ Gasket R45 Octagonal Type Soft Iron Ring Joint to ASME B16.20 High Pressure Service</v>
       </c>
       <c r="C9" t="str">
-        <v>Fasteners</v>
+        <v>Fittings</v>
       </c>
       <c r="D9" t="str">
-        <v>Set</v>
+        <v>Nos</v>
       </c>
       <c r="E9">
-        <v>350</v>
+        <v>1880</v>
       </c>
       <c r="F9">
-        <v>22000</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>BPCL-BLT-ST-2416</v>
+        <v>BPCL-LTG-EXP-200W</v>
       </c>
       <c r="B10" t="str">
-        <v>Stud Bolt M24 x 160mm Long ASTM A193 Grade B7 with 2 Heavy Hex Nuts 2H</v>
+        <v>Explosion-Proof LED Flood Luminaire 200W Ex d IIC T5 IP66 Heavy Duty Weatherproof Refinery Yard Lighting</v>
       </c>
       <c r="C10" t="str">
-        <v>Fasteners</v>
+        <v>Electrical</v>
       </c>
       <c r="D10" t="str">
-        <v>Set</v>
+        <v>Nos</v>
       </c>
       <c r="E10">
-        <v>530</v>
+        <v>34800</v>
       </c>
       <c r="F10">
-        <v>16000</v>
+        <v>390</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>BPCL-BLT-SS-1690</v>
+        <v>BPCL-PPE-GAS-4WAY</v>
       </c>
       <c r="B11" t="str">
-        <v>Stainless Steel Stud Bolt M16 x 90mm Long ASTM A193 B8M with 2 Nuts 8M</v>
+        <v>Four Gas Detector Portable Confined Space Monitor O2/LEL/CO/H2S with Suction Pump &amp; Calibration Kit Ex ia IIC T4</v>
       </c>
       <c r="C11" t="str">
-        <v>Fasteners</v>
+        <v>Safety</v>
       </c>
       <c r="D11" t="str">
-        <v>Set</v>
+        <v>Nos</v>
       </c>
       <c r="E11">
-        <v>790</v>
+        <v>56500</v>
       </c>
       <c r="F11">
-        <v>8200</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>BPCL-FLG-WN-306</v>
+        <v>BPCL-PPE-SCBA-300B</v>
       </c>
       <c r="B12" t="str">
-        <v>Flange WNRF 6 inch 300# Sch 40 Bore CS ASTM A105 ASME B16.5</v>
+        <v>Breathing Apparatus SCBA Set 6.8 Litre Carbon Fibre Cylinder 300 Bar Complete with Harness Mask &amp; Whistle Alarm EN137</v>
       </c>
       <c r="C12" t="str">
-        <v>Fittings</v>
+        <v>Safety</v>
       </c>
       <c r="D12" t="str">
-        <v>Nos</v>
+        <v>Set</v>
       </c>
       <c r="E12">
-        <v>6250</v>
+        <v>82800</v>
       </c>
       <c r="F12">
-        <v>1100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>BPCL-FLG-WN-154</v>
+        <v>BPCL-VAL-CHCK-6300D</v>
       </c>
       <c r="B13" t="str">
-        <v>Flange Weld Neck 4 inch Class 150 Raised Face ASTM A105 ASME B16.5</v>
+        <v>Check Valve Dual Plate Wafer Style 6" 300# Duplex Steel ASTM A890 Gr 4A / UNS S31803 Spring Loaded API 594</v>
       </c>
       <c r="C13" t="str">
-        <v>Fittings</v>
+        <v>Valves</v>
       </c>
       <c r="D13" t="str">
         <v>Nos</v>
       </c>
       <c r="E13">
-        <v>3450</v>
+        <v>52500</v>
       </c>
       <c r="F13">
-        <v>1450</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>BPCL-FIT-ELB-906</v>
+        <v>BPCL-TUB-BOIL-T22</v>
       </c>
       <c r="B14" t="str">
-        <v>Elbow 90 Deg LR 6 inch NB Sch 40 Seamless WPB to ASTM A234 ASME B16.9</v>
+        <v>Tube Boiler Seamless Alloy Steel A213 T22 50.8mm OD (2 Inch) x 4.5mm Min Wall Thickness Heat Exchanger Tubing</v>
       </c>
       <c r="C14" t="str">
-        <v>Fittings</v>
+        <v>Pipes</v>
       </c>
       <c r="D14" t="str">
-        <v>Nos</v>
+        <v>Mtr</v>
       </c>
       <c r="E14">
-        <v>2850</v>
+        <v>3880</v>
       </c>
       <c r="F14">
-        <v>1950</v>
+        <v>4100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>BPCL-GSK-SW-306</v>
+        <v>BPCL-BRG-BALL-6312</v>
       </c>
       <c r="B15" t="str">
-        <v>Gasket Spiral Wound 6 inch 300# SS316/Graphite with Inner/Outer Ring B16.20</v>
+        <v>Bearing Deep Groove Ball 6312-2Z/C3 Double Shield 60 mm Shaft Dia Dynamic Load 85kN SKF Equivalent</v>
       </c>
       <c r="C15" t="str">
-        <v>Fittings</v>
+        <v>Mechanical</v>
       </c>
       <c r="D15" t="str">
         <v>Nos</v>
       </c>
       <c r="E15">
-        <v>460</v>
+        <v>3150</v>
       </c>
       <c r="F15">
-        <v>12500</v>
+        <v>550</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>BPCL-PMP-SEAL-50</v>
+        <v>BPCL-LPG-CAR-CPL-02</v>
       </c>
       <c r="B16" t="str">
-        <v>Cartridge Mechanical Seal 50mm for Centrifugal Process Pump API 682</v>
+        <v>High Flow LPG Carousel Filling Gun Electronic Auto-Shutoff 50 bar Viton Seal</v>
       </c>
       <c r="C16" t="str">
-        <v>Mechanical</v>
+        <v>LPG</v>
       </c>
       <c r="D16" t="str">
         <v>Nos</v>
       </c>
       <c r="E16">
-        <v>43500</v>
+        <v>48500</v>
       </c>
       <c r="F16">
-        <v>95</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>BPCL-LTG-FL-60W</v>
+        <v>BPCL-TRK-BOT-LD-ARM</v>
       </c>
       <c r="B17" t="str">
-        <v>Flameproof Explosion Proof LED Luminaire 60W Zone 1 Gas Group IIA/IIB/IIC</v>
+        <v>Terminal Bottom Loading Arm 4" Counterbalanced with API Coupler &amp; Vapor Recovery Hose</v>
       </c>
       <c r="C17" t="str">
-        <v>Electrical</v>
+        <v>Terminal</v>
       </c>
       <c r="D17" t="str">
         <v>Nos</v>
       </c>
       <c r="E17">
-        <v>18800</v>
+        <v>340000</v>
       </c>
       <c r="F17">
-        <v>750</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>BPCL-PPE-HLM-01</v>
+        <v>BPCL-TNK-ALM-IFR-40</v>
       </c>
       <c r="B18" t="str">
-        <v>Industrial Safety Helmet White Colour with 4-Point Suspension IS:2925</v>
+        <v>Internal Floating Roof (IFR) Full Contact Aluminum Pan Type for 40m Dia Petrol Storage Tank</v>
       </c>
       <c r="C18" t="str">
-        <v>Safety</v>
+        <v>Storage</v>
       </c>
       <c r="D18" t="str">
         <v>Nos</v>
       </c>
       <c r="E18">
-        <v>490</v>
+        <v>2850000</v>
       </c>
       <c r="F18">
-        <v>5500</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>BPCL-PPE-GLV-NIT</v>
+        <v>BPCL-MEC-TURB-MTR-06</v>
       </c>
       <c r="B19" t="str">
-        <v>Nitrile Chemical Gloves Heavy Duty Gauntlet Cuff 13" Green EN388</v>
+        <v>Custody Transfer Turbine Flow Meter 6" Class 300 with Dual Pickoff &amp; Preamplifier for POL</v>
       </c>
       <c r="C19" t="str">
-        <v>Safety</v>
+        <v>Terminal</v>
       </c>
       <c r="D19" t="str">
-        <v>Pair</v>
+        <v>Nos</v>
       </c>
       <c r="E19">
-        <v>330</v>
+        <v>420000</v>
       </c>
       <c r="F19">
-        <v>11000</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>BPCL-REF-STM-TRP</v>
+        <v>BPCL-SAF-FOAM-PROP</v>
       </c>
       <c r="B20" t="str">
-        <v>Thermodynamic Steam Trap 1/2" NPT Class 600 Forged Carbon Steel Body</v>
+        <v>Balanced Pressure Foam Proportioner Skid 1000 LPM with Concentrate Tank &amp; Deluge Valve</v>
       </c>
       <c r="C20" t="str">
-        <v>Mechanical</v>
+        <v>Safety</v>
       </c>
       <c r="D20" t="str">
         <v>Nos</v>
       </c>
       <c r="E20">
-        <v>5400</v>
+        <v>680000</v>
       </c>
       <c r="F20">
-        <v>650</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>BPCL-LPG-LOAD-ARM</v>
+        <v>BPCL-RETAIL-DISP-MPD</v>
       </c>
       <c r="B21" t="str">
-        <v>LPG Bottom Loading Coupler 4" API RP 1004 Cam-and-Groove with Viton Seals</v>
+        <v>Multi-Product Fuel Dispenser (MPD) 4-Hose Dual Sided with Electronic Volume Totalizer &amp; POS Interface</v>
       </c>
       <c r="C21" t="str">
-        <v>Refinery</v>
+        <v>Retail</v>
       </c>
       <c r="D21" t="str">
         <v>Nos</v>
       </c>
       <c r="E21">
-        <v>88000</v>
+        <v>460000</v>
       </c>
       <c r="F21">
-        <v>35</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>